<commit_message>
Ottimizzazione tempo con BeautifulSoup
</commit_message>
<xml_diff>
--- a/btp_dati.xlsx
+++ b/btp_dati.xlsx
@@ -428,7 +428,7 @@
   <dimension ref="A1:M160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="121" customWidth="1" min="1" max="1"/>
     <col width="33" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -513,12 +513,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>IT0001086567</t>
+          <t>IT0001086567 -Btp-1nv26      7,25%Ultimo: 106,31Cedola: 3,625Scadenza: 01/11/2026IT0001086567</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Btp-1nv26 7,25%</t>
+          <t>Btp-1nv26      7,25%</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -560,12 +560,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>IT0001174611</t>
+          <t>IT0001174611 -Btp-1nv27       6,5%Ultimo: 109,37Cedola: 3,25Scadenza: 01/11/2027IT0001174611</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Btp-1nv27 6,5%</t>
+          <t>Btp-1nv27       6,5%</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -607,12 +607,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>IT0001278511</t>
+          <t>IT0001278511 -Btp-1nv29      5,25%Ultimo: 111,14Cedola: 2,625Scadenza: 01/11/2029IT0001278511</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Btp-1nv29 5,25%</t>
+          <t>Btp-1nv29      5,25%</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -654,12 +654,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>IT0001444378</t>
+          <t>IT0001444378 -Btp-1mg31         6%Ultimo: 117,05Cedola: 3,00Scadenza: 01/05/2031IT0001444378</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Btp-1mg31 6%</t>
+          <t>Btp-1mg31         6%</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -701,12 +701,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>IT0003256820</t>
+          <t>IT0003256820 -Btp-1fb33      5,75%Ultimo: 117,44Cedola: 2,875Scadenza: 01/02/2033IT0003256820</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Btp-1fb33 5,75%</t>
+          <t>Btp-1fb33      5,75%</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -748,12 +748,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>IT0003535157</t>
+          <t>IT0003535157 -Btp-1ag34         5%Ultimo: 113,20Cedola: 2,50Scadenza: 01/08/2034IT0003535157</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Btp-1ag34 5%</t>
+          <t>Btp-1ag34         5%</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -795,12 +795,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>IT0003745541</t>
+          <t>IT0003745541 -Btpi-15st35    2,35%Ultimo: 108,13Cedola: 1,175Scadenza: 15/09/2035IT0003745541</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Btpi-15st35 2,35%</t>
+          <t>Btpi-15st35    2,35%</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -842,12 +842,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>IT0003934657</t>
+          <t>IT0003934657 -Btp-1fb37         4%Ultimo: 104,34Cedola: 2,00Scadenza: 01/02/2037IT0003934657</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Btp-1fb37 4%</t>
+          <t>Btp-1fb37         4%</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -889,12 +889,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>IT0004286966</t>
+          <t>IT0004286966 -Btp-1ag39         5%Ultimo: 113,50Cedola: 2,50Scadenza: 01/08/2039IT0004286966</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Btp-1ag39 5%</t>
+          <t>Btp-1ag39         5%</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -936,7 +936,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>IT0004532559</t>
+          <t>IT0004532559 -Btp-1st40 5%Ultimo: 113,26Cedola: 2,50Scadenza: 01/09/2040IT0004532559</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>IT0004545890</t>
+          <t>IT0004545890 -Btpi-15st41 2,55%Ultimo: 107,78Cedola: 1,275Scadenza: 15/09/2041IT0004545890</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1030,7 +1030,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>IT0004644735</t>
+          <t>IT0004644735 -Btp-1mz26 4,5%Ultimo: 101,368Cedola: 2,25Scadenza: 01/03/2026IT0004644735</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1077,7 +1077,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>IT0004735152</t>
+          <t>IT0004735152 -Btpi-15st26 3,1%Ultimo: 103,00Cedola: 1,55Scadenza: 15/09/2026IT0004735152</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1124,7 +1124,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>IT0004848443</t>
+          <t>IT0004848443 -Btp Coupon Strip Zc Nv26 EurUltimo: 97,87Cedola:Scadenza: 01/11/2026IT0004848443</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1147,7 +1147,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>IT0004848476</t>
+          <t>IT0004848476 -Btp Coupon Strip Zc Nv27 EurUltimo: 95,49Cedola:Scadenza: 01/11/2027IT0004848476</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1170,7 +1170,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>IT0004848484</t>
+          <t>IT0004848484 -Btp Coupon Strip Zc Nv29 EurUltimo: 90,42Cedola:Scadenza: 01/11/2029IT0004848484</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1193,7 +1193,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>IT0004848492</t>
+          <t>IT0004848492 -Btp Coupon Strip Zc Mg31 EurUltimo: 85,68Cedola:Scadenza: 01/05/2031IT0004848492</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1216,7 +1216,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>IT0004848534</t>
+          <t>IT0004848534 -Btpstripital Zc Feb33 EurUltimo: 79,57Cedola:Scadenza: 01/02/2033IT0004848534</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1239,7 +1239,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>IT0004848641</t>
+          <t>IT0004848641 -Btpstripital Zc Feb37 EurUltimo:Cedola:Scadenza: 01/02/2037IT0004848641</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1259,7 +1259,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>IT0004848690</t>
+          <t>IT0004848690 -Btpstripital Zc Ago39Ultimo:Cedola:Scadenza: 01/08/2039IT0004848690</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1279,7 +1279,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>IT0004889033</t>
+          <t>IT0004889033 -Btp Tf 4,75% St28 EurUltimo: 107,17Cedola: 2,375Scadenza: 01/09/2028IT0004889033</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1326,7 +1326,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>IT0004923998</t>
+          <t>IT0004923998 -Btp Tf 4,75% St44 EurUltimo: 109,78Cedola: 2,375Scadenza: 01/09/2044IT0004923998</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1373,7 +1373,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>IT0004976525</t>
+          <t>IT0004976525 -Btp Coupon Strip Zc St28 EurUltimo: 93,41Cedola:Scadenza: 01/09/2028IT0004976525</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1396,7 +1396,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>IT0004976558</t>
+          <t>IT0004976558 -Btp Coupon Strip Zc Mz30 EurUltimo: 89,16Cedola:Scadenza: 01/03/2030IT0004976558</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1419,7 +1419,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>IT0004976590</t>
+          <t>IT0004976590 -Btpstripital Zc Mar32Ultimo: 83,11Cedola:Scadenza: 01/03/2032IT0004976590</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1442,7 +1442,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>IT0004976632</t>
+          <t>IT0004976632 -Btpstripital Zc Mar34Ultimo:Cedola:Scadenza: 01/03/2034IT0004976632</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1462,7 +1462,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>IT0004976657</t>
+          <t>IT0004976657 -Btpstripital Zc Mar35 EurUltimo:Cedola:Scadenza: 01/03/2035IT0004976657</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1482,7 +1482,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>IT0004976681</t>
+          <t>IT0004976681 -Btpstripital Zc Sep36 EurUltimo:Cedola:Scadenza: 01/09/2036IT0004976681</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1502,7 +1502,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>IT0004976715</t>
+          <t>IT0004976715 -Btpstripital Zc Mar38Ultimo: 62,47Cedola:Scadenza: 01/03/2038IT0004976715</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1525,7 +1525,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>IT0005024234</t>
+          <t>IT0005024234 -Btp Tf 3,50% Mz30 EurUltimo: 104,03Cedola: 1,75Scadenza: 01/03/2030IT0005024234</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1572,7 +1572,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>IT0005083057</t>
+          <t>IT0005083057 -Btp Tf 3,25% St46 EurUltimo: 88,26Cedola: 1,625Scadenza: 01/09/2046IT0005083057</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1619,7 +1619,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>IT0005094088</t>
+          <t>IT0005094088 -Btp Tf 1,65% Mz32 EurUltimo: 92,38Cedola: 0,825Scadenza: 01/03/2032IT0005094088</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1666,7 +1666,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>IT0005127086</t>
+          <t>IT0005127086 -Btp Tf 2,00% Dc25 EurUltimo: 100,007Cedola: 1,00Scadenza: 01/12/2025IT0005127086</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1713,7 +1713,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>IT0005138828</t>
+          <t>IT0005138828 -Btpi Tf 1,25% St32 EurUltimo: 100,28Cedola: 0,625Scadenza: 15/09/2032IT0005138828</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1760,7 +1760,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>IT0005162828</t>
+          <t>IT0005162828 -Btp Tf 2,7% Mz47 EurUltimo: 80,33Cedola: 1,35Scadenza: 01/03/2047IT0005162828</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1807,7 +1807,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>IT0005170839</t>
+          <t>IT0005170839 -Btp Tf 1,60% Gn26 EurUltimo: 99,727Cedola: 0,80Scadenza: 01/06/2026IT0005170839</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1854,7 +1854,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>IT0005177909</t>
+          <t>IT0005177909 -Btp Tf 2,25% St36 EurUltimo: 88,43Cedola: 1,125Scadenza: 01/09/2036IT0005177909</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1901,7 +1901,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>IT0005210650</t>
+          <t>IT0005210650 -Btp Tf 1.25% Dc26 EurUltimo: 99,14Cedola: 0,625Scadenza: 01/12/2026IT0005210650</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1948,7 +1948,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>IT0005217390</t>
+          <t>IT0005217390 -Btp Tf 2,8% Mz67 EurUltimo: 71,49Cedola: 1,40Scadenza: 01/03/2067IT0005217390</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1995,7 +1995,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>IT0005240350</t>
+          <t>IT0005240350 -Btp Tf 2,45% St33 EurUltimo: 95,04Cedola: 1,225Scadenza: 01/09/2033IT0005240350</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2042,7 +2042,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>IT0005240830</t>
+          <t>IT0005240830 -Btp Tf 2,20% Gn27 EurUltimo: 100,29Cedola: 1,10Scadenza: 01/06/2027IT0005240830</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2089,7 +2089,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>IT0005246134</t>
+          <t>IT0005246134 -Btpi Tf 1,30% Mg28 EurUltimo:Cedola: 0,65Scadenza: 15/05/2028IT0005246134</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2118,7 +2118,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>IT0005273013</t>
+          <t>IT0005273013 -Btp Tf 3,45% Mz48 EurUltimo: 90,32Cedola: 1,725Scadenza: 01/03/2048IT0005273013</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2165,7 +2165,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>IT0005274805</t>
+          <t>IT0005274805 -Btp Tf 2,05% Ag27 EurUltimo: 99,95Cedola: 1,025Scadenza: 01/08/2027IT0005274805</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2212,7 +2212,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>IT0005321325</t>
+          <t>IT0005321325 -Btp Tf 2,95% St38 EurUltimo: 92,32Cedola: 1,475Scadenza: 01/09/2038IT0005321325</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2259,7 +2259,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>IT0005323032</t>
+          <t>IT0005323032 -Btp Tf 2,00% Fb28 EurUltimo: 99,63Cedola: 1,00Scadenza: 01/02/2028IT0005323032</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2306,7 +2306,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>IT0005332835</t>
+          <t>IT0005332835 -Btp Italia Mg26 EurUltimo: 99,90Cedola: 0,275Scadenza: 21/05/2026IT0005332835</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2353,7 +2353,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>IT0005340929</t>
+          <t>IT0005340929 -Btp Tf 2,80% Dc28 EurUltimo: 101,55Cedola: 1,40Scadenza: 01/12/2028IT0005340929</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2400,7 +2400,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>IT0005345183</t>
+          <t>IT0005345183 -Btp Tf 2.50% Nv25 EurUltimo: 100,116Cedola: 1,25Scadenza: 15/11/2025IT0005345183</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>IT0005358806</t>
+          <t>IT0005358806 -Btp Tf 3,35% Mz35 EurUltimo: 100,06Cedola: 1,675Scadenza: 01/03/2035IT0005358806</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2494,7 +2494,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>IT0005363111</t>
+          <t>IT0005363111 -Btp Tf 3,85% St49 EurUltimo: 95,50Cedola: 1,925Scadenza: 01/09/2049IT0005363111</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2541,7 +2541,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>IT0005365165</t>
+          <t>IT0005365165 -Btp Tf 3,00% Ag29 EurUltimo: 102,10Cedola: 1,50Scadenza: 01/08/2029IT0005365165</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2588,7 +2588,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>IT0005370306</t>
+          <t>IT0005370306 -Btp Tf 2,10% Lg26 EurUltimo: 100,106Cedola: 1,05Scadenza: 15/07/2026IT0005370306</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2635,7 +2635,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>IT0005377152</t>
+          <t>IT0005377152 -Btp Tf 3,1% Mz40 EurUltimo: 92,09Cedola: 1,55Scadenza: 01/03/2040IT0005377152</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2682,7 +2682,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>IT0005383309</t>
+          <t>IT0005383309 -Btp Tf 1,35% Ap30 EurUltimo: 94,68Cedola: 0,675Scadenza: 01/04/2030IT0005383309</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2729,7 +2729,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>IT0005387052</t>
+          <t>IT0005387052 -Btpi Tf 0,4% Mg30 EurUltimo: 97,38Cedola: 0,20Scadenza: 15/05/2030IT0005387052</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2776,7 +2776,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>IT0005388175</t>
+          <t>IT0005388175 -Btp Italia Ot27 EurUltimo: 99,88Cedola: 0,325Scadenza: 28/10/2027IT0005388175</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2823,7 +2823,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>IT0005390874</t>
+          <t>IT0005390874 -Btp Tf 0,85% Ge27 EurUltimo: 98,43Cedola: 0,425Scadenza: 15/01/2027IT0005390874</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2870,7 +2870,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>IT0005398406</t>
+          <t>IT0005398406 -Btp Tf 2,45% St50 EurUltimo: 73,43Cedola: 1,225Scadenza: 01/09/2050IT0005398406</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2917,7 +2917,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>IT0005402117</t>
+          <t>IT0005402117 -Btp Tf 1,45% Mz36 EurUltimo: 82,06Cedola: 0,725Scadenza: 01/03/2036IT0005402117</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2964,7 +2964,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>IT0005403396</t>
+          <t>IT0005403396 -Btp Tf 0,95% Ag30 EurUltimo: 92,11Cedola: 0,475Scadenza: 01/08/2030IT0005403396</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3011,7 +3011,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>IT0005413171</t>
+          <t>IT0005413171 -Btp Tf 1,65% Dc30 EurUltimo: 94,69Cedola: 0,825Scadenza: 01/12/2030IT0005413171</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3058,7 +3058,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>IT0005415291</t>
+          <t>IT0005415291 -Btp Futura Lg30 EurUltimo: 94,01Cedola: 0,65Scadenza: 14/07/2030IT0005415291</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3105,7 +3105,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>IT0005415416</t>
+          <t>IT0005415416 -Btpi Tf 0,65% Mg26 EurUltimo:Cedola: 0,325Scadenza: 15/05/2026IT0005415416</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3134,7 +3134,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>IT0005416570</t>
+          <t>IT0005416570 -Btp Tf 0,95% St27 EurUltimo: 97,68Cedola: 0,475Scadenza: 15/09/2027IT0005416570</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3181,7 +3181,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>IT0005419848</t>
+          <t>IT0005419848 -Btp Tf 0,50% Fb26 EurUltimo: 99,31Cedola: 0,25Scadenza: 01/02/2026IT0005419848</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3228,7 +3228,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>IT0005421703</t>
+          <t>IT0005421703 -Btp Tf 1,8% Mz41 EurUltimo: 75,76Cedola: 0,90Scadenza: 01/03/2041IT0005421703</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3275,7 +3275,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>IT0005422891</t>
+          <t>IT0005422891 -Btp Tf 0,90% Ap31 EurUltimo: 90,18Cedola: 0,45Scadenza: 01/04/2031IT0005422891</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3322,7 +3322,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>IT0005425233</t>
+          <t>IT0005425233 -Btp Tf 1,7% St51 EurUltimo: 61,64Cedola: 0,85Scadenza: 01/09/2051IT0005425233</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3369,7 +3369,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>IT0005425761</t>
+          <t>IT0005425761 -Btp Futura Nv28 EurUltimo: 95,41Cedola: 0,30Scadenza: 17/11/2028IT0005425761</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3416,7 +3416,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>IT0005433195</t>
+          <t>IT0005433195 -Btp Tf 0,95% Mz37 EurUltimo: 75,25Cedola: 0,475Scadenza: 01/03/2037IT0005433195</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3463,7 +3463,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>IT0005433690</t>
+          <t>IT0005433690 -Btp Tf 0,25% Mz28 EurUltimo: 95,14Cedola: 0,125Scadenza: 15/03/2028IT0005433690</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3510,7 +3510,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>IT0005436693</t>
+          <t>IT0005436693 -Btp Tf 0,6% Ag31 EurUltimo: 87,75Cedola: 0,30Scadenza: 01/08/2031IT0005436693</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3557,7 +3557,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>IT0005436701</t>
+          <t>IT0005436701 -Btpi Tf 0,15% Mg51 EurUltimo: 61,09Cedola: 0,075Scadenza: 15/05/2051IT0005436701</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3604,7 +3604,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>IT0005437147</t>
+          <t>IT0005437147 -Btp Tf 0% Ap26 EurUltimo: 98,794Cedola:Scadenza: 01/04/2026IT0005437147</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -3627,7 +3627,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>IT0005438004</t>
+          <t>IT0005438004 -Btpgreen 1,5%Ap45eurUltimo: 66,23Cedola: 0,75Scadenza: 30/04/2045IT0005438004</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -3674,7 +3674,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>IT0005441883</t>
+          <t>IT0005441883 -Btp Tf 2,15% Mz72 EurUltimo: 58,70Cedola: 1,075Scadenza: 01/03/2072IT0005441883</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -3721,7 +3721,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>IT0005442097</t>
+          <t>IT0005442097 -Btp Futura Ap37 EurUltimo: 79,30Cedola: 0,60Scadenza: 27/04/2037IT0005442097</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -3768,7 +3768,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>IT0005445306</t>
+          <t>IT0005445306 -Btp Tf 0,5% Lg28 EurUltimo: 95,05Cedola: 0,25Scadenza: 15/07/2028IT0005445306</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -3815,7 +3815,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>IT0005449969</t>
+          <t>IT0005449969 -Btp Tf 0,95% Dc31 EurUltimo: 88,85Cedola: 0,475Scadenza: 01/12/2031IT0005449969</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -3862,7 +3862,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>IT0005454241</t>
+          <t>IT0005454241 -Btp Tf 0% Ag26 EurUltimo: 98,272Cedola:Scadenza: 01/08/2026IT0005454241</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -3885,7 +3885,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>IT0005466013</t>
+          <t>IT0005466013 -Btp Tf 0,95% Gn32 EurUltimo: 87,61Cedola: 0,475Scadenza: 01/06/2032IT0005466013</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -3932,7 +3932,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>IT0005466351</t>
+          <t>IT0005466351 -Btp Futura Nv33 EurUltimo: 87,53Cedola: 0,375Scadenza: 16/11/2033IT0005466351</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -3979,7 +3979,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>IT0005467482</t>
+          <t>IT0005467482 -Btp Tf 0,45% Fb29 EurUltimo: 93,51Cedola: 0,225Scadenza: 15/02/2029IT0005467482</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -4026,7 +4026,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>IT0005480980</t>
+          <t>IT0005480980 -Btp Tf 2,15% St52 EurUltimo: 67,47Cedola: 1,075Scadenza: 01/09/2052IT0005480980</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -4073,7 +4073,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>IT0005482994</t>
+          <t>IT0005482994 -Btpi Tf 0,1% Mg33 EurUltimo: 90,42Cedola: 0,05Scadenza: 15/05/2033IT0005482994</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -4120,7 +4120,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>IT0005484552</t>
+          <t>IT0005484552 -Btp Tf 1,1% Ap27 EurUltimo: 98,45Cedola: 0,55Scadenza: 01/04/2027IT0005484552</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -4167,7 +4167,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>IT0005493298</t>
+          <t>IT0005493298 -Btp Tf 1,2% Ag25 EurUltimo: 99,989Cedola: 0,60Scadenza: 15/08/2025IT0005493298</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -4214,7 +4214,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>IT0005494239</t>
+          <t>IT0005494239 -Btp Tf 2,5% Dc32 EurUltimo: 96,37Cedola: 1,25Scadenza: 01/12/2032IT0005494239</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -4261,7 +4261,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>IT0005495731</t>
+          <t>IT0005495731 -Btp Tf 2,80% Gn29 EurUltimo: 101,20Cedola: 1,40Scadenza: 15/06/2029IT0005495731</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4308,7 +4308,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>IT0005496770</t>
+          <t>IT0005496770 -Btp Tf 3,25% Mz38 EurUltimo: 95,72Cedola: 1,625Scadenza: 01/03/2038IT0005496770</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -4355,7 +4355,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>IT0005497000</t>
+          <t>IT0005497000 -Btp Italia Gn30 EurUltimo: 101,10Cedola: 0,80Scadenza: 28/06/2030IT0005497000</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -4402,7 +4402,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>IT0005498685</t>
+          <t>IT0005498685 -Btpstripital Zc Dec25 EurUltimo:Cedola:Scadenza: 15/12/2025IT0005498685</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -4422,7 +4422,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>IT0005498693</t>
+          <t>IT0005498693 -Btpstripital Zc Jun26 EurUltimo:Cedola:Scadenza: 15/06/2026IT0005498693</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -4442,7 +4442,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>IT0005498701</t>
+          <t>IT0005498701 -Btpstripital Zc Dec26 EurUltimo:Cedola:Scadenza: 15/12/2026IT0005498701</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -4462,7 +4462,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>IT0005498719</t>
+          <t>IT0005498719 -Btpstripital Zc Jun27 EurUltimo:Cedola:Scadenza: 15/06/2027IT0005498719</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4482,7 +4482,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>IT0005498727</t>
+          <t>IT0005498727 -Btpstripital Zc Dec27 EurUltimo:Cedola:Scadenza: 15/12/2027IT0005498727</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -4502,7 +4502,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>IT0005498735</t>
+          <t>IT0005498735 -Btpstripital Zc Jun28 EurUltimo:Cedola:Scadenza: 15/06/2028IT0005498735</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -4522,7 +4522,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>IT0005498743</t>
+          <t>IT0005498743 -Btpstripital Zc Dec28 EurUltimo:Cedola:Scadenza: 15/12/2028IT0005498743</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -4542,7 +4542,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>IT0005498750</t>
+          <t>IT0005498750 -Btpstripital Zc Jun29 EurUltimo:Cedola:Scadenza: 15/06/2029IT0005498750</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -4562,7 +4562,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>IT0005500068</t>
+          <t>IT0005500068 -Btp Tf 2,65% Dc27 EurUltimo: 101,04Cedola: 1,325Scadenza: 01/12/2027IT0005500068</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -4609,7 +4609,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>IT0005508590</t>
+          <t>IT0005508590 -Btpgreen 4%Ap35eurUltimo: 105,67Cedola: 2,00Scadenza: 30/04/2035IT0005508590</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -4656,7 +4656,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>IT0005514473</t>
+          <t>IT0005514473 -Btp Tf 3,5% Ge26 EurUltimo: 100,627Cedola: 1,75Scadenza: 15/01/2026IT0005514473</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -4703,7 +4703,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>IT0005517195</t>
+          <t>IT0005517195 -Btp Italia Nv28 EurUltimo: 101,60Cedola: 0,80Scadenza: 22/11/2028IT0005517195</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -4750,7 +4750,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>IT0005518128</t>
+          <t>IT0005518128 -Btp Tf 4,40% Mg33 EurUltimo: 108,63Cedola: 2,20Scadenza: 01/05/2033IT0005518128</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -4797,7 +4797,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>IT0005519787</t>
+          <t>IT0005519787 -Btp Tf 3,85% Dc29 EurUltimo: 105,18Cedola: 1,925Scadenza: 15/12/2029IT0005519787</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -4844,7 +4844,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>IT0005521981</t>
+          <t>IT0005521981 -Btp Tf 3,4% Ap28 EurUltimo: 102,91Cedola: 1,70Scadenza: 01/04/2028IT0005521981</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -4891,7 +4891,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>IT0005526162</t>
+          <t>IT0005526162 -Btpstripital Zc Dec29 EurUltimo:Cedola:Scadenza: 15/12/2029IT0005526162</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -4911,7 +4911,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>IT0005530032</t>
+          <t>IT0005530032 -Btp Tf 4,45% St43 EurUltimo: 105,36Cedola: 2,225Scadenza: 01/09/2043IT0005530032</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -4958,7 +4958,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>IT0005532723</t>
+          <t>IT0005532723 -Btp Italia Mz28 EurUltimo: 102,42Cedola: 1,00Scadenza: 14/03/2028IT0005532723</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -5005,7 +5005,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>IT0005534141</t>
+          <t>IT0005534141 -Btp Tf 4,5% Ot53 EurUltimo: 103,12Cedola: 2,25Scadenza: 01/10/2053IT0005534141</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -5052,7 +5052,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>IT0005538597</t>
+          <t>IT0005538597 -Btp Tf 3,80% Ap26 EurUltimo: 101,19Cedola: 1,90Scadenza: 15/04/2026IT0005538597</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -5099,7 +5099,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>IT0005542359</t>
+          <t>IT0005542359 -Btpgreen 4%Ot31eurUltimo: 106,49Cedola: 2,00Scadenza: 30/10/2031IT0005542359</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -5146,7 +5146,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>IT0005542797</t>
+          <t>IT0005542797 -Btp Tf 3,7% Gn30 EurUltimo: 104,61Cedola: 1,85Scadenza: 15/06/2030IT0005542797</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -5193,7 +5193,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>IT0005543803</t>
+          <t>IT0005543803 -Btpi Tf 1.5% Mg29 EurUltimo: 101,96Cedola: 0,75Scadenza: 15/05/2029IT0005543803</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -5240,7 +5240,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>IT0005544082</t>
+          <t>IT0005544082 -Btp Tf 4,35% Nv33 EurUltimo: 108,16Cedola: 2,175Scadenza: 01/11/2033IT0005544082</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -5287,7 +5287,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>IT0005547408</t>
+          <t>IT0005547408 -Btp Valore Gn27 EurUltimo: 102,87Cedola: 2,00Scadenza: 13/06/2027IT0005547408</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -5334,7 +5334,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>IT0005547812</t>
+          <t>IT0005547812 -Btpi Tf 2,4% Mg39 EurUltimo: 104,30Cedola: 1,20Scadenza: 15/05/2039IT0005547812</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -5381,7 +5381,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>IT0005548315</t>
+          <t>IT0005548315 -Btp Tf 3,8% Ag28 EurUltimo: 104,24Cedola: 1,90Scadenza: 01/08/2028IT0005548315</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -5428,7 +5428,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>IT0005550204</t>
+          <t>IT0005550204 -Btpstripital Zc Ott39Ultimo: 57,85Cedola:Scadenza: 01/10/2039IT0005550204</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -5451,7 +5451,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>IT0005556011</t>
+          <t>IT0005556011 -Btp Tf 3,85% St26 EurUltimo: 101,89Cedola: 1,925Scadenza: 15/09/2026IT0005556011</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -5498,7 +5498,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>IT0005557084</t>
+          <t>IT0005557084 -Btp Tf 3,6% St25 EurUltimo: 100,202Cedola: 1,80Scadenza: 29/09/2025IT0005557084</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -5545,7 +5545,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>IT0005560948</t>
+          <t>IT0005560948 -Btp Tf 4,2% Mz34 EurUltimo: 107,00Cedola: 2,10Scadenza: 01/03/2034IT0005560948</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -5592,7 +5592,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>IT0005561888</t>
+          <t>IT0005561888 -Btp Fx 4% Nov30 EurUltimo: 106,02Cedola: 2,00Scadenza: 15/11/2030IT0005561888</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -5639,7 +5639,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>IT0005565400</t>
+          <t>IT0005565400 -Btp Valore Sc Oct28 EurUltimo: 105,15Cedola: 1,025Scadenza: 10/10/2028IT0005565400</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -5686,7 +5686,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>IT0005566408</t>
+          <t>IT0005566408 -Btp Fx 4.1% Feb29 EurUltimo: 105,55Cedola:Scadenza: 01/02/2029IT0005566408</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -5709,7 +5709,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>IT0005580045</t>
+          <t>IT0005580045 -Btp Fx 2.95% Feb27 EurUltimo: 101,21Cedola: 1,475Scadenza: 15/02/2027IT0005580045</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -5756,7 +5756,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>IT0005580094</t>
+          <t>IT0005580094 -Btp Fx 3.5% Feb31 EurUltimo: 103,47Cedola: 1,75Scadenza: 15/02/2031IT0005580094</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -5803,7 +5803,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>IT0005582421</t>
+          <t>IT0005582421 -Btp Fx 4.15% Oct39 EurUltimo: 103,70Cedola:Scadenza: 01/10/2039IT0005582421</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -5826,7 +5826,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>IT0005583486</t>
+          <t>IT0005583486 -Btp Valore Sc Mz30 EurUltimo: 103,74Cedola: 0,8125Scadenza: 05/03/2030IT0005583486</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -5873,7 +5873,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>IT0005584302</t>
+          <t>IT0005584302 -Btp Fx 3.2% Jan26 EurUltimo: 100,516Cedola: 1,60Scadenza: 28/01/2026IT0005584302</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -5920,7 +5920,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>IT0005584849</t>
+          <t>IT0005584849 -Btp Fx 3.35% Jul29 EurUltimo: 103,08Cedola: 1,675Scadenza: 01/07/2029IT0005584849</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -5967,7 +5967,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>IT0005584856</t>
+          <t>IT0005584856 -Btp Fx 3.85% Jul34 EurUltimo: 104,19Cedola: 1,925Scadenza: 01/07/2034IT0005584856</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -6014,7 +6014,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>IT0005588881</t>
+          <t>IT0005588881 -Btpi Fx May36 EurUltimo: 99,87Cedola: 0,90Scadenza: 15/05/2036IT0005588881</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -6061,7 +6061,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>IT0005594483</t>
+          <t>IT0005594483 -Btp Valore Sc Mg30 EurUltimo: 103,67Cedola: 0,8375Scadenza: 14/05/2030IT0005594483</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -6108,7 +6108,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>IT0005595803</t>
+          <t>IT0005595803 -Btp Fx 3.45% Jul31 EurUltimo: 103,02Cedola: 1,725Scadenza: 15/07/2031IT0005595803</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -6155,7 +6155,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>IT0005596470</t>
+          <t>IT0005596470 -Btp Green Fx 4.05% Oct37 EurUltimo: 104,12Cedola: 2,025Scadenza: 30/10/2037IT0005596470</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -6202,7 +6202,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>IT0005599904</t>
+          <t>IT0005599904 -Btp Fx 3.45% Jul27 EurUltimo: 102,45Cedola: 1,725Scadenza: 15/07/2027IT0005599904</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -6249,7 +6249,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>IT0005607269</t>
+          <t>IT0005607269 -Btp Fx 3.1% Aug26 EurUltimo: 101,06Cedola: 1,55Scadenza: 28/08/2026IT0005607269</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -6296,7 +6296,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>IT0005607970</t>
+          <t>IT0005607970 -Btp Fx 3.85% Feb35 EurUltimo: 103,78Cedola: 1,925Scadenza: 01/02/2035IT0005607970</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -6343,7 +6343,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>IT0005611055</t>
+          <t>IT0005611055 -Btp Fx 3% Oct29 EurUltimo: 102,20Cedola: 1,50Scadenza: 01/10/2029IT0005611055</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -6390,7 +6390,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>IT0005611741</t>
+          <t>IT0005611741 -Btp Fx 4.3% Oct54 EurUltimo: 99,23Cedola: 2,15Scadenza: 01/10/2054IT0005611741</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -6437,7 +6437,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>IT0005619546</t>
+          <t>IT0005619546 -Btp Fx 3.15% Nov31 EurUltimo: 101,17Cedola: 1,575Scadenza: 15/11/2031IT0005619546</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -6484,7 +6484,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>IT0005622128</t>
+          <t>IT0005622128 -Btp Fx 2.7% Oct27 EurUltimo: 101,07Cedola: 1,35Scadenza: 15/10/2027IT0005622128</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -6531,7 +6531,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>IT0005631590</t>
+          <t>IT0005631590 -Btp Fx 3.65% Aug35 EurUltimo: 101,69Cedola: 1,825Scadenza: 01/08/2035IT0005631590</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -6578,7 +6578,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>IT0005631608</t>
+          <t>IT0005631608 -Btp Green Fx 4.1% Apr46 EurUltimo: 100,66Cedola: 2,05Scadenza: 30/04/2046IT0005631608</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -6625,7 +6625,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>IT0005633794</t>
+          <t>IT0005633794 -Btp Fx 2.55% Feb27 EurUltimo: 100,68Cedola: 1,275Scadenza: 25/02/2027IT0005633794</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -6672,7 +6672,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>IT0005634800</t>
+          <t>IT0005634800 -Btp Piu' Sc Fb33 EurUltimo: 100,74Cedola: 0,7125Scadenza: 25/02/2033IT0005634800</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -6719,7 +6719,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>IT0005635583</t>
+          <t>IT0005635583 -Btp Fx 3.85% Oct40 EurUltimo: 99,50Cedola: 1,925Scadenza: 01/10/2040IT0005635583</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -6766,7 +6766,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>IT0005637399</t>
+          <t>IT0005637399 -Btp Fx 2.95% Jul30 EurUltimo: 101,14Cedola: 1,475Scadenza: 01/07/2030IT0005637399</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -6813,7 +6813,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>IT0005641029</t>
+          <t>IT0005641029 -Btp Fx 2.65% Jun28 EurUltimo: 100,93Cedola: 1,325Scadenza: 15/06/2028IT0005641029</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -6860,7 +6860,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>IT0005647265</t>
+          <t>IT0005647265 -Btp Fx 3.25% Jul32 EurUltimo: 101,23Cedola: 1,625Scadenza: 15/07/2032IT0005647265</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -6907,7 +6907,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>IT0005647273</t>
+          <t>IT0005647273 -Btpi Fx May56 EurUltimo: 101,38Cedola: 1,275Scadenza: 15/05/2056IT0005647273</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -6954,7 +6954,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>IT0005648149</t>
+          <t>IT0005648149 -Btp Fx 3.6% Oct35 EurUltimo: 101,10Cedola: 1,49508Scadenza: 01/10/2035IT0005648149</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -7001,7 +7001,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>IT0005648255</t>
+          <t>IT0005648255 -Btp Italia Jun32 EurUltimo: 100,73Cedola: 0,925Scadenza: 04/06/2032IT0005648255</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -7048,7 +7048,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>IT0005654642</t>
+          <t>IT0005654642 -Btp Fx 2.7% Oct30 EurUltimo: 99,71Cedola: 0,82623Scadenza: 01/10/2030IT0005654642</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -7095,7 +7095,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>IT0005657330</t>
+          <t>IT0005657330 -Btp Fx 2.1% Aug27 EurUltimo: 99,85Cedola: 0,34807Scadenza: 26/08/2027IT0005657330</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -7142,7 +7142,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>IT0005657348</t>
+          <t>IT0005657348 -Btpi Fx Aug31 EurUltimo: 99,70Cedola: 0,1489Scadenza: 15/08/2031IT0005657348</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -7189,7 +7189,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>IT0005660052</t>
+          <t>IT0005660052 -Btp Fx 2.35% Jan29 EurUltimo: 99,70Cedola: 1,175Scadenza: 15/01/2029IT0005660052</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">

</xml_diff>

<commit_message>
Modifiche finali 25 ago 25
</commit_message>
<xml_diff>
--- a/btp_dati.xlsx
+++ b/btp_dati.xlsx
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>106.19</v>
+        <v>106.1</v>
       </c>
       <c r="D2" t="n">
         <v>3.625</v>
@@ -497,7 +497,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>109.25</v>
+        <v>109.11</v>
       </c>
       <c r="D3" t="n">
         <v>3.25</v>
@@ -520,7 +520,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>111</v>
+        <v>110.61</v>
       </c>
       <c r="D4" t="n">
         <v>2.625</v>
@@ -543,7 +543,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>116.87</v>
+        <v>116.49</v>
       </c>
       <c r="D5" t="n">
         <v>3</v>
@@ -566,7 +566,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>117.2</v>
+        <v>116.8</v>
       </c>
       <c r="D6" t="n">
         <v>2.875</v>
@@ -589,7 +589,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>112.81</v>
+        <v>112.38</v>
       </c>
       <c r="D7" t="n">
         <v>2.5</v>
@@ -612,7 +612,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>107.17</v>
+        <v>106.79</v>
       </c>
       <c r="D8" t="n">
         <v>1.175</v>
@@ -635,7 +635,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>103.72</v>
+        <v>103.19</v>
       </c>
       <c r="D9" t="n">
         <v>2</v>
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>112.55</v>
+        <v>111.95</v>
       </c>
       <c r="D10" t="n">
         <v>2.5</v>
@@ -681,7 +681,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>112.37</v>
+        <v>111.73</v>
       </c>
       <c r="D11" t="n">
         <v>2.5</v>
@@ -704,7 +704,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>106.15</v>
+        <v>105.4</v>
       </c>
       <c r="D12" t="n">
         <v>1.275</v>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>101.271</v>
+        <v>101.253</v>
       </c>
       <c r="D13" t="n">
         <v>2.25</v>
@@ -749,6 +749,9 @@
           <t>Btpi-15st26 3,1%</t>
         </is>
       </c>
+      <c r="C14" t="n">
+        <v>102.86</v>
+      </c>
       <c r="D14" t="n">
         <v>1.55</v>
       </c>
@@ -790,7 +793,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>95.56</v>
+        <v>95.47</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -810,7 +813,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>90.41</v>
+        <v>90.22</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -830,7 +833,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>85.2</v>
+        <v>85.25</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -901,7 +904,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>107.07</v>
+        <v>106.87</v>
       </c>
       <c r="D22" t="n">
         <v>2.375</v>
@@ -924,7 +927,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>108.62</v>
+        <v>107.85</v>
       </c>
       <c r="D23" t="n">
         <v>2.375</v>
@@ -947,7 +950,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>93.42</v>
+        <v>93.37</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -967,7 +970,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>89.26000000000001</v>
+        <v>89.06999999999999</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1072,7 +1075,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>104.05</v>
+        <v>103.78</v>
       </c>
       <c r="D31" t="n">
         <v>1.75</v>
@@ -1095,7 +1098,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>87.2</v>
+        <v>86.51000000000001</v>
       </c>
       <c r="D32" t="n">
         <v>1.625</v>
@@ -1118,7 +1121,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>92.29000000000001</v>
+        <v>91.97</v>
       </c>
       <c r="D33" t="n">
         <v>0.825</v>
@@ -1141,7 +1144,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>100.01</v>
+        <v>100</v>
       </c>
       <c r="D34" t="n">
         <v>1</v>
@@ -1164,7 +1167,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>100.03</v>
+        <v>99.70999999999999</v>
       </c>
       <c r="D35" t="n">
         <v>0.625</v>
@@ -1187,7 +1190,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>79.23999999999999</v>
+        <v>78.51000000000001</v>
       </c>
       <c r="D36" t="n">
         <v>1.35</v>
@@ -1210,7 +1213,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>99.736</v>
+        <v>99.729</v>
       </c>
       <c r="D37" t="n">
         <v>0.8</v>
@@ -1233,7 +1236,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>88.06</v>
+        <v>87.58</v>
       </c>
       <c r="D38" t="n">
         <v>1.125</v>
@@ -1256,7 +1259,7 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>99.14</v>
+        <v>99.06</v>
       </c>
       <c r="D39" t="n">
         <v>0.625</v>
@@ -1279,7 +1282,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>69.83</v>
+        <v>69.11</v>
       </c>
       <c r="D40" t="n">
         <v>1.4</v>
@@ -1302,7 +1305,7 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>94.81999999999999</v>
+        <v>94.31999999999999</v>
       </c>
       <c r="D41" t="n">
         <v>1.225</v>
@@ -1325,7 +1328,7 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>100.27</v>
+        <v>100.2</v>
       </c>
       <c r="D42" t="n">
         <v>1.1</v>
@@ -1348,7 +1351,7 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>101.19</v>
+        <v>101.25</v>
       </c>
       <c r="D43" t="n">
         <v>0.65</v>
@@ -1371,7 +1374,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>89.09999999999999</v>
+        <v>88.43000000000001</v>
       </c>
       <c r="D44" t="n">
         <v>1.725</v>
@@ -1394,7 +1397,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>99.95</v>
+        <v>99.87</v>
       </c>
       <c r="D45" t="n">
         <v>1.025</v>
@@ -1417,7 +1420,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>91.7</v>
+        <v>91.18000000000001</v>
       </c>
       <c r="D46" t="n">
         <v>1.475</v>
@@ -1440,7 +1443,7 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>99.56</v>
+        <v>99.54000000000001</v>
       </c>
       <c r="D47" t="n">
         <v>1</v>
@@ -1463,7 +1466,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>99.836</v>
+        <v>99.84999999999999</v>
       </c>
       <c r="D48" t="n">
         <v>0.275</v>
@@ -1486,7 +1489,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>101.55</v>
+        <v>101.43</v>
       </c>
       <c r="D49" t="n">
         <v>1.4</v>
@@ -1509,7 +1512,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>100.099</v>
+        <v>100.078</v>
       </c>
       <c r="D50" t="n">
         <v>1.25</v>
@@ -1532,7 +1535,7 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>99.7</v>
+        <v>99.19</v>
       </c>
       <c r="D51" t="n">
         <v>1.675</v>
@@ -1555,7 +1558,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>94.25</v>
+        <v>93.5</v>
       </c>
       <c r="D52" t="n">
         <v>1.925</v>
@@ -1578,7 +1581,7 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>102.06</v>
+        <v>101.85</v>
       </c>
       <c r="D53" t="n">
         <v>1.5</v>
@@ -1601,7 +1604,7 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>100.1</v>
+        <v>100.071</v>
       </c>
       <c r="D54" t="n">
         <v>1.05</v>
@@ -1624,7 +1627,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>91.33</v>
+        <v>90.73</v>
       </c>
       <c r="D55" t="n">
         <v>1.55</v>
@@ -1647,7 +1650,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>94.66</v>
+        <v>94.45999999999999</v>
       </c>
       <c r="D56" t="n">
         <v>0.675</v>
@@ -1670,7 +1673,7 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>97.23</v>
+        <v>97.12</v>
       </c>
       <c r="D57" t="n">
         <v>0.2</v>
@@ -1693,7 +1696,7 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>99.81</v>
+        <v>99.79000000000001</v>
       </c>
       <c r="D58" t="n">
         <v>0.325</v>
@@ -1716,7 +1719,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>98.45</v>
+        <v>98.5</v>
       </c>
       <c r="D59" t="n">
         <v>0.425</v>
@@ -1739,7 +1742,7 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>72.22</v>
+        <v>71.67</v>
       </c>
       <c r="D60" t="n">
         <v>1.225</v>
@@ -1762,7 +1765,7 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>81.69</v>
+        <v>81.27</v>
       </c>
       <c r="D61" t="n">
         <v>0.725</v>
@@ -1785,7 +1788,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>92.09</v>
+        <v>91.86</v>
       </c>
       <c r="D62" t="n">
         <v>0.475</v>
@@ -1808,7 +1811,7 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>94.66</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="D63" t="n">
         <v>0.825</v>
@@ -1831,7 +1834,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>93.94</v>
+        <v>93.7</v>
       </c>
       <c r="D64" t="n">
         <v>0.65</v>
@@ -1854,7 +1857,7 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>99.59399999999999</v>
+        <v>99.521</v>
       </c>
       <c r="D65" t="n">
         <v>0.325</v>
@@ -1877,7 +1880,7 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>97.72</v>
+        <v>97.65000000000001</v>
       </c>
       <c r="D66" t="n">
         <v>0.475</v>
@@ -1900,7 +1903,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>99.364</v>
+        <v>99.348</v>
       </c>
       <c r="D67" t="n">
         <v>0.25</v>
@@ -1923,7 +1926,7 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>74.98</v>
+        <v>74.48999999999999</v>
       </c>
       <c r="D68" t="n">
         <v>0.9</v>
@@ -1946,7 +1949,7 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>90.17</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="D69" t="n">
         <v>0.45</v>
@@ -1969,7 +1972,7 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>60.43</v>
+        <v>59.88</v>
       </c>
       <c r="D70" t="n">
         <v>0.85</v>
@@ -1992,7 +1995,7 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>95.23</v>
+        <v>95.26000000000001</v>
       </c>
       <c r="D71" t="n">
         <v>0.3</v>
@@ -2015,7 +2018,7 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>74.78</v>
+        <v>74.34</v>
       </c>
       <c r="D72" t="n">
         <v>0.475</v>
@@ -2038,7 +2041,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>95.20999999999999</v>
+        <v>95.08</v>
       </c>
       <c r="D73" t="n">
         <v>0.125</v>
@@ -2061,7 +2064,7 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>87.73999999999999</v>
+        <v>87.47</v>
       </c>
       <c r="D74" t="n">
         <v>0.3</v>
@@ -2084,7 +2087,7 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>58.73</v>
+        <v>58.13</v>
       </c>
       <c r="D75" t="n">
         <v>0.075</v>
@@ -2107,7 +2110,7 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>98.84099999999999</v>
+        <v>98.821</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2127,7 +2130,7 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>65.26000000000001</v>
+        <v>64.72</v>
       </c>
       <c r="D77" t="n">
         <v>0.75</v>
@@ -2150,7 +2153,7 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>57.49</v>
+        <v>56.85</v>
       </c>
       <c r="D78" t="n">
         <v>1.075</v>
@@ -2173,7 +2176,7 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>79.09999999999999</v>
+        <v>78.77</v>
       </c>
       <c r="D79" t="n">
         <v>0.6</v>
@@ -2196,7 +2199,7 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>95.13</v>
+        <v>94.98999999999999</v>
       </c>
       <c r="D80" t="n">
         <v>0.25</v>
@@ -2219,7 +2222,7 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>88.78</v>
+        <v>88.48999999999999</v>
       </c>
       <c r="D81" t="n">
         <v>0.475</v>
@@ -2242,7 +2245,7 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>98.29900000000001</v>
+        <v>98.268</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2262,7 +2265,7 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>87.54000000000001</v>
+        <v>87.19</v>
       </c>
       <c r="D83" t="n">
         <v>0.475</v>
@@ -2285,7 +2288,7 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>87.3</v>
+        <v>86.91</v>
       </c>
       <c r="D84" t="n">
         <v>0.375</v>
@@ -2308,7 +2311,7 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>93.62</v>
+        <v>93.5</v>
       </c>
       <c r="D85" t="n">
         <v>0.225</v>
@@ -2331,7 +2334,7 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>66.05</v>
+        <v>65.47</v>
       </c>
       <c r="D86" t="n">
         <v>1.075</v>
@@ -2354,7 +2357,7 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>90.02</v>
+        <v>89.70999999999999</v>
       </c>
       <c r="D87" t="n">
         <v>0.05</v>
@@ -2377,7 +2380,7 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>98.53</v>
+        <v>98.45</v>
       </c>
       <c r="D88" t="n">
         <v>0.55</v>
@@ -2400,7 +2403,7 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>96.19</v>
+        <v>95.81</v>
       </c>
       <c r="D89" t="n">
         <v>1.25</v>
@@ -2423,7 +2426,7 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>101.19</v>
+        <v>101.01</v>
       </c>
       <c r="D90" t="n">
         <v>1.4</v>
@@ -2446,7 +2449,7 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>95.06999999999999</v>
+        <v>94.5</v>
       </c>
       <c r="D91" t="n">
         <v>1.625</v>
@@ -2469,7 +2472,7 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>100.86</v>
+        <v>100.8</v>
       </c>
       <c r="D92" t="n">
         <v>0.8</v>
@@ -2628,7 +2631,7 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>101.05</v>
+        <v>100.91</v>
       </c>
       <c r="D101" t="n">
         <v>1.325</v>
@@ -2651,7 +2654,7 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>105.27</v>
+        <v>104.77</v>
       </c>
       <c r="D102" t="n">
         <v>2</v>
@@ -2674,7 +2677,7 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>100.549</v>
+        <v>100.544</v>
       </c>
       <c r="D103" t="n">
         <v>1.75</v>
@@ -2697,7 +2700,7 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>101.51</v>
+        <v>101.42</v>
       </c>
       <c r="D104" t="n">
         <v>0.8</v>
@@ -2720,7 +2723,7 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>108.37</v>
+        <v>107.99</v>
       </c>
       <c r="D105" t="n">
         <v>2.2</v>
@@ -2743,7 +2746,7 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>105.11</v>
+        <v>104.88</v>
       </c>
       <c r="D106" t="n">
         <v>1.925</v>
@@ -2766,7 +2769,7 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>102.89</v>
+        <v>102.78</v>
       </c>
       <c r="D107" t="n">
         <v>1.7</v>
@@ -2806,7 +2809,7 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>104.33</v>
+        <v>103.69</v>
       </c>
       <c r="D109" t="n">
         <v>2.225</v>
@@ -2829,7 +2832,7 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>102.43</v>
+        <v>102.34</v>
       </c>
       <c r="D110" t="n">
         <v>1</v>
@@ -2852,7 +2855,7 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>101.48</v>
+        <v>100.63</v>
       </c>
       <c r="D111" t="n">
         <v>2.25</v>
@@ -2875,7 +2878,7 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>101.126</v>
+        <v>101.11</v>
       </c>
       <c r="D112" t="n">
         <v>1.9</v>
@@ -2898,7 +2901,7 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>106.27</v>
+        <v>106.02</v>
       </c>
       <c r="D113" t="n">
         <v>2</v>
@@ -2921,7 +2924,7 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>104.53</v>
+        <v>104.28</v>
       </c>
       <c r="D114" t="n">
         <v>1.85</v>
@@ -2943,9 +2946,6 @@
           <t>Btpi Tf 1.5% Mg29 Eur</t>
         </is>
       </c>
-      <c r="C115" t="n">
-        <v>101.9</v>
-      </c>
       <c r="D115" t="n">
         <v>0.75</v>
       </c>
@@ -2967,7 +2967,7 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>107.84</v>
+        <v>107.39</v>
       </c>
       <c r="D116" t="n">
         <v>2.175</v>
@@ -2990,7 +2990,7 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>102.95</v>
+        <v>102.81</v>
       </c>
       <c r="D117" t="n">
         <v>2</v>
@@ -3013,7 +3013,7 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>103.1</v>
+        <v>102.68</v>
       </c>
       <c r="D118" t="n">
         <v>1.2</v>
@@ -3036,7 +3036,7 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>104.19</v>
+        <v>104.04</v>
       </c>
       <c r="D119" t="n">
         <v>1.9</v>
@@ -3076,7 +3076,7 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>101.86</v>
+        <v>101.79</v>
       </c>
       <c r="D121" t="n">
         <v>1.925</v>
@@ -3099,7 +3099,7 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>100.144</v>
+        <v>100.15</v>
       </c>
       <c r="D122" t="n">
         <v>1.8</v>
@@ -3122,7 +3122,7 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>106.64</v>
+        <v>106.17</v>
       </c>
       <c r="D123" t="n">
         <v>2.1</v>
@@ -3145,7 +3145,7 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>105.92</v>
+        <v>105.61</v>
       </c>
       <c r="D124" t="n">
         <v>2</v>
@@ -3168,7 +3168,7 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>105.45</v>
+        <v>105.17</v>
       </c>
       <c r="D125" t="n">
         <v>1.025</v>
@@ -3191,7 +3191,7 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>105.47</v>
+        <v>105.28</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3211,7 +3211,7 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>101.17</v>
+        <v>101.14</v>
       </c>
       <c r="D127" t="n">
         <v>1.475</v>
@@ -3234,7 +3234,7 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>103.34</v>
+        <v>103.06</v>
       </c>
       <c r="D128" t="n">
         <v>1.75</v>
@@ -3257,7 +3257,7 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>102.95</v>
+        <v>102.28</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3277,7 +3277,7 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>103.78</v>
+        <v>103.55</v>
       </c>
       <c r="D130" t="n">
         <v>0.8125</v>
@@ -3300,7 +3300,7 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>100.491</v>
+        <v>100.467</v>
       </c>
       <c r="D131" t="n">
         <v>1.6</v>
@@ -3323,7 +3323,7 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>103.01</v>
+        <v>102.81</v>
       </c>
       <c r="D132" t="n">
         <v>1.675</v>
@@ -3346,7 +3346,7 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>103.81</v>
+        <v>103.38</v>
       </c>
       <c r="D133" t="n">
         <v>1.925</v>
@@ -3369,7 +3369,7 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>98.98</v>
+        <v>98.7</v>
       </c>
       <c r="D134" t="n">
         <v>0.9</v>
@@ -3392,7 +3392,7 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>103.7</v>
+        <v>103.36</v>
       </c>
       <c r="D135" t="n">
         <v>0.8375</v>
@@ -3415,7 +3415,7 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>102.91</v>
+        <v>102.64</v>
       </c>
       <c r="D136" t="n">
         <v>1.725</v>
@@ -3438,7 +3438,7 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>103.44</v>
+        <v>102.86</v>
       </c>
       <c r="D137" t="n">
         <v>2.025</v>
@@ -3461,7 +3461,7 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>102.31</v>
+        <v>102.28</v>
       </c>
       <c r="D138" t="n">
         <v>1.725</v>
@@ -3484,7 +3484,7 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>101.06</v>
+        <v>101</v>
       </c>
       <c r="D139" t="n">
         <v>1.55</v>
@@ -3507,7 +3507,7 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>103.36</v>
+        <v>102.9</v>
       </c>
       <c r="D140" t="n">
         <v>1.925</v>
@@ -3530,7 +3530,7 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>101.68</v>
+        <v>101.48</v>
       </c>
       <c r="D141" t="n">
         <v>1.5</v>
@@ -3553,7 +3553,7 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>97.62</v>
+        <v>96.84999999999999</v>
       </c>
       <c r="D142" t="n">
         <v>2.15</v>
@@ -3576,7 +3576,7 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>101.04</v>
+        <v>100.71</v>
       </c>
       <c r="D143" t="n">
         <v>1.575</v>
@@ -3599,7 +3599,7 @@
         </is>
       </c>
       <c r="C144" t="n">
-        <v>100.11</v>
+        <v>100.97</v>
       </c>
       <c r="D144" t="n">
         <v>1.35</v>
@@ -3622,7 +3622,7 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>101.29</v>
+        <v>100.78</v>
       </c>
       <c r="D145" t="n">
         <v>1.825</v>
@@ -3645,7 +3645,7 @@
         </is>
       </c>
       <c r="C146" t="n">
-        <v>99.39</v>
+        <v>98.7</v>
       </c>
       <c r="D146" t="n">
         <v>2.05</v>
@@ -3668,7 +3668,7 @@
         </is>
       </c>
       <c r="C147" t="n">
-        <v>100.59</v>
+        <v>100.58</v>
       </c>
       <c r="D147" t="n">
         <v>1.275</v>
@@ -3691,7 +3691,7 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>100.77</v>
+        <v>100.44</v>
       </c>
       <c r="D148" t="n">
         <v>0.7125</v>
@@ -3714,7 +3714,7 @@
         </is>
       </c>
       <c r="C149" t="n">
-        <v>98.66</v>
+        <v>98.08</v>
       </c>
       <c r="D149" t="n">
         <v>1.925</v>
@@ -3737,7 +3737,7 @@
         </is>
       </c>
       <c r="C150" t="n">
-        <v>100.91</v>
+        <v>100.82</v>
       </c>
       <c r="D150" t="n">
         <v>1.475</v>
@@ -3760,7 +3760,7 @@
         </is>
       </c>
       <c r="C151" t="n">
-        <v>100.83</v>
+        <v>100.81</v>
       </c>
       <c r="D151" t="n">
         <v>1.325</v>
@@ -3783,7 +3783,7 @@
         </is>
       </c>
       <c r="C152" t="n">
-        <v>100.94</v>
+        <v>100.69</v>
       </c>
       <c r="D152" t="n">
         <v>1.625</v>
@@ -3806,7 +3806,7 @@
         </is>
       </c>
       <c r="C153" t="n">
-        <v>98.38</v>
+        <v>97.3</v>
       </c>
       <c r="D153" t="n">
         <v>1.275</v>
@@ -3829,7 +3829,7 @@
         </is>
       </c>
       <c r="C154" t="n">
-        <v>100.64</v>
+        <v>100.18</v>
       </c>
       <c r="D154" t="n">
         <v>1.49508</v>
@@ -3852,7 +3852,7 @@
         </is>
       </c>
       <c r="C155" t="n">
-        <v>100.47</v>
+        <v>100.29</v>
       </c>
       <c r="D155" t="n">
         <v>0.925</v>
@@ -3875,7 +3875,7 @@
         </is>
       </c>
       <c r="C156" t="n">
-        <v>99.69</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="D156" t="n">
         <v>0.82623</v>
@@ -3898,7 +3898,7 @@
         </is>
       </c>
       <c r="C157" t="n">
-        <v>99.94</v>
+        <v>99.93000000000001</v>
       </c>
       <c r="D157" t="n">
         <v>0.34807</v>
@@ -3921,7 +3921,7 @@
         </is>
       </c>
       <c r="C158" t="n">
-        <v>99.38</v>
+        <v>99.36</v>
       </c>
       <c r="D158" t="n">
         <v>0.55</v>
@@ -3944,7 +3944,7 @@
         </is>
       </c>
       <c r="C159" t="n">
-        <v>99.75</v>
+        <v>99.56</v>
       </c>
       <c r="D159" t="n">
         <v>1.175</v>

</xml_diff>